<commit_message>
Update DMN.xlsx: swap Cowl num_rows/num_stitches formulas (rows=measurement-based, stitches=fixed constant)
</commit_message>
<xml_diff>
--- a/DMN.xlsx
+++ b/DMN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f7e89476d29c7cb/Documents/GitHub/pcp_manager/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_F29E6D4A3312D0E33A46B6F415544F871D815D97" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94F7F8F5-E3A8-4E3B-AED8-B19FC6D518FE}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_F29E6D4A3312D0E33A46B6F415544F871D815D97" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D34B7A7B-C0DF-41CE-A5CE-A49193BAA3F9}"/>
   <bookViews>
     <workbookView xWindow="22944" yWindow="0" windowWidth="23232" windowHeight="18576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -125,16 +125,16 @@
     <t>Default to Not Found</t>
   </si>
   <si>
-    <t>(rows_per_4inch/4)*(4.2*2.75)</t>
-  </si>
-  <si>
-    <t>(stitches_per_4inch/4)*((measurement/3.2)*3.14)</t>
-  </si>
-  <si>
     <t>"Default 0"</t>
   </si>
   <si>
-    <t>"4.2 in = Average Female Nape to Chin measurement | 2.75 = Multiplier for appropriate cowl length | 3.2 = Ratio of cross back to female neck width | 3.14 = Factor to convert neck width to neck circumference. | Note: stitches and rows rversed due to knitting direction"</t>
+    <t>(rows_per_4inch/4)*((measurement/3.2)*3.14)</t>
+  </si>
+  <si>
+    <t>(stitches_per_4inch/4)*(4.2*3.75)</t>
+  </si>
+  <si>
+    <t>"4.2 in = Average Female Nape to Chin measurement | 3.75 = Multiplier for appropriate cowl length | 3.2 = Ratio of cross back to female neck width | 3.14 = Factor to convert neck width to neck circumference."</t>
   </si>
 </sst>
 </file>
@@ -526,14 +526,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -863,10 +863,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="26"/>
+      <c r="C2" s="28"/>
     </row>
     <row r="3" spans="2:3" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
@@ -1017,10 +1017,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="26"/>
     </row>
     <row r="3" spans="2:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
@@ -1093,13 +1093,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" spans="2:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
@@ -1147,7 +1147,7 @@
         <v>30</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I4" s="20" t="s">
         <v>32</v>
@@ -1177,7 +1177,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="21" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="10:10" x14ac:dyDescent="0.3">

</xml_diff>